<commit_message>
Re-ran work from home job increase
</commit_message>
<xml_diff>
--- a/TravelDemandModel/2026_Housing_EIS/Forecast/SocioEcon_2050_Summary_ByScenario.xlsx
+++ b/TravelDemandModel/2026_Housing_EIS/Forecast/SocioEcon_2050_Summary_ByScenario.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SocioEcon_2050_Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income_Pct_by_Scenario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SocioEcon_2050_Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income_Pct_by_Scenario" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -54,10 +54,10 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -441,65 +441,70 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="F1" s="1" t="inlineStr">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Absolute Difference</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>% Difference</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>scenario_1_sum</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>scenario_2_sum</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>scenario_3_sum</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>scenario_4_sum</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>diff_2_vs_1</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>diff_3_vs_1</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>diff_4_vs_1</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>4</v>
       </c>
     </row>
@@ -969,27 +974,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>income_category</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_1</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>scenario_2</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>scenario_3</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>scenario_4</t>
         </is>

</xml_diff>

<commit_message>
Lots of modifications to the scenario config
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/TravelDemandModel/2026_Housing_EIS/Forecast/SocioEcon_2050_Summary_ByScenario.xlsx
+++ b/TravelDemandModel/2026_Housing_EIS/Forecast/SocioEcon_2050_Summary_ByScenario.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11151</v>
+        <v>11147</v>
       </c>
       <c r="C5" t="n">
         <v>13076</v>
@@ -607,13 +607,13 @@
         <v>11354</v>
       </c>
       <c r="F5" t="n">
-        <v>1925</v>
+        <v>1929</v>
       </c>
       <c r="G5" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="H5" t="n">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="I5" s="3">
         <f>F5/$B5</f>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5071</v>
+        <v>5070</v>
       </c>
       <c r="C6" t="n">
         <v>6362</v>
@@ -647,13 +647,13 @@
         <v>5384</v>
       </c>
       <c r="F6" t="n">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="G6" t="n">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="H6" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="I6" s="3">
         <f>F6/$B6</f>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9881</v>
+        <v>9899</v>
       </c>
       <c r="C7" t="n">
         <v>11661</v>
@@ -687,13 +687,13 @@
         <v>9975</v>
       </c>
       <c r="F7" t="n">
-        <v>1780</v>
+        <v>1762</v>
       </c>
       <c r="G7" t="n">
-        <v>1631</v>
+        <v>1613</v>
       </c>
       <c r="H7" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="I7" s="3">
         <f>F7/$B7</f>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.4271922767497989</v>
+        <v>0.4268264665339256</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>0.4204636805041963</v>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.1942688579856721</v>
+        <v>0.1941338642977485</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0.204572494292421</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.378538865264529</v>
+        <v>0.3790396691683259</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0.3749638252033827</v>

</xml_diff>